<commit_message>
update bank management project
</commit_message>
<xml_diff>
--- a/static/fund_transfer_list.xlsx
+++ b/static/fund_transfer_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,6 +441,25 @@
         <is>
           <t>amount</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>197156669267</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fund_transfer</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>20000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>